<commit_message>
Direction : BMC V5, suppression de l'onglet « Changements V3 → V4 » (28/10/2026)
</commit_message>
<xml_diff>
--- a/1 DIRECTION/STRATEGIE/2026 1028 Business Model Canvas V5 - Pop Tables.xlsx
+++ b/1 DIRECTION/STRATEGIE/2026 1028 Business Model Canvas V5 - Pop Tables.xlsx
@@ -8,7 +8,6 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Business Model Canvas" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hypothèses et owners" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Changements V3 → V4" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -1337,252 +1336,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
-  <cols>
-    <col width="20" customWidth="1" style="13" min="1" max="1"/>
-    <col width="46" customWidth="1" style="13" min="2" max="2"/>
-    <col width="58" customWidth="1" style="13" min="3" max="3"/>
-    <col width="40" customWidth="1" style="13" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="17" customHeight="1" s="13">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Ce qui change entre le BMC V3 (28/10, 17 h 24) et le BMC V4 (28/10, soir) : décisions de la Direction</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Bloc</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>V3 (28/10, 17 h 24)</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>V4 (28/10, soir)</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Décision</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="34" customHeight="1" s="13">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Positionnement</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>« Fou d'un soir » (nom de travail) ; triple rareté</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Pop Tables ; segment luxe ; licence propre ; personnel fourni</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>D-02, D-03, D-07, D-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1" s="13">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Proposition de valeur</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Unicité ; convives sélectionnés</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Unicité ; rareté par ville ; accès au moment du drop</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>D-12, D-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="34" customHeight="1" s="13">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Segments</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>5 segments ; séquencement à arbitrer</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Place à l'unité (B2C) ; privatisation (B2C groupes constitués, B2B) ; prescripteurs</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>D-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1" s="13">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Revenus</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Prix affichés à la liste privée ; jauges à recalibrer</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Prix fixes par offre et créneau, sans devis, connus à la réservation ; jauges du fichier Finance</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>D-05, D-10, D-11, D-13</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="34" customHeight="1" s="13">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Relations clients</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Liste privée, Passeport, contrats cadres</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Drop, accès prioritaire de la liste privée, contrats cadres</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>D-12</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="34" customHeight="1" s="13">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Canaux</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Liste privée, concierges, Instagram sans prix, soirée de lancement non budgétée</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Drops sans prix public, site à 15 000 €, soirée de lancement budgétée</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>D-11, D-12, D-14, D-19</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1" s="13">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Partenaires clés</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Associé gastronomique en option</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Associé gastronomique validé (equity in kind) ; investisseurs financiers ; partenaires locaux par ville</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>D-17, D-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="34" customHeight="1" s="13">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Activités clés</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>1 soirée ouverte par mois ; montage de licence à trancher</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>1 soirée à la place par mois et par ville ; 1 → 3 → 6 villes ; licence propre</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>D-09, D-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="34" customHeight="1" s="13">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Structure de coûts</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Équipe S3 ; photographe ; rentabilité dépendante des jauges</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Équipe à 15–20 % du CA ; pas de photographe ; site, lancement, licence, ouvertures de villes</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>D-06, D-08, D-14, D-19</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0"/>
-</worksheet>
 </file>
</xml_diff>